<commit_message>
Direct Write Excel for QC-21 Day 5
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-21.xlsx
+++ b/FM-MN-07_QC-21.xlsx
@@ -1752,7 +1752,11 @@
       <c r="D6" s="22" t="inlineStr"/>
       <c r="E6" s="22" t="inlineStr"/>
       <c r="F6" s="22" t="inlineStr"/>
-      <c r="G6" s="22" t="inlineStr"/>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H6" s="22" t="inlineStr"/>
       <c r="I6" s="22" t="inlineStr"/>
       <c r="J6" s="22" t="inlineStr"/>
@@ -1793,7 +1797,11 @@
       <c r="D7" s="22" t="inlineStr"/>
       <c r="E7" s="22" t="inlineStr"/>
       <c r="F7" s="22" t="inlineStr"/>
-      <c r="G7" s="22" t="inlineStr"/>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H7" s="22" t="inlineStr"/>
       <c r="I7" s="22" t="inlineStr"/>
       <c r="J7" s="22" t="inlineStr"/>
@@ -1834,7 +1842,11 @@
       <c r="D8" s="22" t="inlineStr"/>
       <c r="E8" s="22" t="inlineStr"/>
       <c r="F8" s="22" t="inlineStr"/>
-      <c r="G8" s="22" t="inlineStr"/>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H8" s="22" t="inlineStr"/>
       <c r="I8" s="22" t="inlineStr"/>
       <c r="J8" s="22" t="inlineStr"/>
@@ -1875,7 +1887,11 @@
       <c r="D9" s="22" t="inlineStr"/>
       <c r="E9" s="22" t="inlineStr"/>
       <c r="F9" s="22" t="inlineStr"/>
-      <c r="G9" s="22" t="inlineStr"/>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H9" s="22" t="inlineStr"/>
       <c r="I9" s="22" t="inlineStr"/>
       <c r="J9" s="22" t="inlineStr"/>
@@ -1916,7 +1932,11 @@
       <c r="D10" s="22" t="inlineStr"/>
       <c r="E10" s="22" t="inlineStr"/>
       <c r="F10" s="22" t="inlineStr"/>
-      <c r="G10" s="22" t="inlineStr"/>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H10" s="22" t="inlineStr"/>
       <c r="I10" s="22" t="inlineStr"/>
       <c r="J10" s="22" t="inlineStr"/>
@@ -1951,7 +1971,11 @@
       <c r="D11" s="38" t="inlineStr"/>
       <c r="E11" s="38" t="inlineStr"/>
       <c r="F11" s="38" t="inlineStr"/>
-      <c r="G11" s="38" t="inlineStr"/>
+      <c r="G11" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ไพรัตน์ </t>
+        </is>
+      </c>
       <c r="H11" s="38" t="inlineStr"/>
       <c r="I11" s="38" t="inlineStr"/>
       <c r="J11" s="38" t="inlineStr"/>
@@ -2089,7 +2113,11 @@
       </c>
     </row>
     <row r="16" ht="185.25" customHeight="1">
-      <c r="B16" s="41" t="inlineStr"/>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>[วันที่ 5]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="23.25" customHeight="1"/>
     <row r="18" ht="21" customHeight="1">
@@ -2135,8 +2163,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Direct Write Excel for QC-21 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-21.xlsx
+++ b/FM-MN-07_QC-21.xlsx
@@ -1757,7 +1757,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="H6" s="22" t="inlineStr"/>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="22" t="inlineStr"/>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
@@ -1802,7 +1806,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="H7" s="22" t="inlineStr"/>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I7" s="22" t="inlineStr"/>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
@@ -1847,7 +1855,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="H8" s="22" t="inlineStr"/>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I8" s="22" t="inlineStr"/>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
@@ -1892,7 +1904,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr"/>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I9" s="22" t="inlineStr"/>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
@@ -1937,7 +1953,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="H10" s="22" t="inlineStr"/>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="22" t="inlineStr"/>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
@@ -1976,7 +1996,11 @@
           <t xml:space="preserve">ไพรัตน์ </t>
         </is>
       </c>
-      <c r="H11" s="38" t="inlineStr"/>
+      <c r="H11" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ไพรัตน์ </t>
+        </is>
+      </c>
       <c r="I11" s="38" t="inlineStr"/>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
@@ -2115,7 +2139,7 @@
     <row r="16" ht="185.25" customHeight="1">
       <c r="B16" s="41" t="inlineStr">
         <is>
-          <t>[วันที่ 5]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ</t>
+          <t>[วันที่ 5]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ,  [วันที่ 6]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ, ข้อ 4: ส่งสอบเทียบ</t>
         </is>
       </c>
     </row>
@@ -2163,8 +2187,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-21 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-21.xlsx
+++ b/FM-MN-07_QC-21.xlsx
@@ -1765,7 +1765,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr"/>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
       <c r="L6" s="22" t="inlineStr"/>
@@ -1814,7 +1818,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I7" s="22" t="inlineStr"/>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr"/>
@@ -1863,7 +1871,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr"/>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
       <c r="L8" s="22" t="inlineStr"/>
@@ -1912,7 +1924,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I9" s="22" t="inlineStr"/>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
       <c r="L9" s="22" t="inlineStr"/>
@@ -1961,7 +1977,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr"/>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
       <c r="L10" s="22" t="inlineStr"/>
@@ -2004,7 +2024,11 @@
           <t xml:space="preserve">ไพรัตน์ </t>
         </is>
       </c>
-      <c r="I11" s="38" t="inlineStr"/>
+      <c r="I11" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ไพรัตน์ </t>
+        </is>
+      </c>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
       <c r="L11" s="38" t="inlineStr"/>
@@ -2146,7 +2170,7 @@
     <row r="16" ht="185.25" customHeight="1">
       <c r="B16" s="41" t="inlineStr">
         <is>
-          <t>[วันที่ 5]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ,  [วันที่ 6]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ, ข้อ 4: ส่งสอบเทียบ</t>
+          <t>[วันที่ 5]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ,  [วันที่ 6]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบ, ข้อ 4: ส่งสอบเทียบ,  [วันที่ 7]: ข้อ 2: ส่งสอบเทียบ, ข้อ 3: ส่งสอบเทียบส่งสอบเทียบ</t>
         </is>
       </c>
     </row>
@@ -2194,8 +2218,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-21 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-21.xlsx
+++ b/FM-MN-07_QC-21.xlsx
@@ -1772,7 +1772,11 @@
       </c>
       <c r="J6" s="22" t="inlineStr"/>
       <c r="K6" s="22" t="inlineStr"/>
-      <c r="L6" s="22" t="inlineStr"/>
+      <c r="L6" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="22" t="inlineStr"/>
       <c r="N6" s="22" t="inlineStr"/>
       <c r="O6" s="22" t="inlineStr"/>
@@ -1825,7 +1829,11 @@
       </c>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr"/>
-      <c r="L7" s="22" t="inlineStr"/>
+      <c r="L7" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="22" t="inlineStr"/>
       <c r="N7" s="22" t="inlineStr"/>
       <c r="O7" s="22" t="inlineStr"/>
@@ -1878,7 +1886,11 @@
       </c>
       <c r="J8" s="22" t="inlineStr"/>
       <c r="K8" s="22" t="inlineStr"/>
-      <c r="L8" s="22" t="inlineStr"/>
+      <c r="L8" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="22" t="inlineStr"/>
       <c r="N8" s="22" t="inlineStr"/>
       <c r="O8" s="22" t="inlineStr"/>
@@ -1931,7 +1943,11 @@
       </c>
       <c r="J9" s="22" t="inlineStr"/>
       <c r="K9" s="22" t="inlineStr"/>
-      <c r="L9" s="22" t="inlineStr"/>
+      <c r="L9" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="22" t="inlineStr"/>
       <c r="N9" s="22" t="inlineStr"/>
       <c r="O9" s="22" t="inlineStr"/>
@@ -1984,7 +2000,11 @@
       </c>
       <c r="J10" s="22" t="inlineStr"/>
       <c r="K10" s="22" t="inlineStr"/>
-      <c r="L10" s="22" t="inlineStr"/>
+      <c r="L10" s="22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="22" t="inlineStr"/>
       <c r="N10" s="22" t="inlineStr"/>
       <c r="O10" s="22" t="inlineStr"/>
@@ -2031,7 +2051,11 @@
       </c>
       <c r="J11" s="38" t="inlineStr"/>
       <c r="K11" s="38" t="inlineStr"/>
-      <c r="L11" s="38" t="inlineStr"/>
+      <c r="L11" s="40" t="inlineStr">
+        <is>
+          <t>ปวีณ์กร</t>
+        </is>
+      </c>
       <c r="M11" s="38" t="inlineStr"/>
       <c r="N11" s="38" t="inlineStr"/>
       <c r="O11" s="38" t="inlineStr"/>
@@ -2218,8 +2242,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>